<commit_message>
fix: stabilize API-05 OpenAI candidate ranking
</commit_message>
<xml_diff>
--- a/docs/specs/whereisit-api-spec-v2.xlsx
+++ b/docs/specs/whereisit-api-spec-v2.xlsx
@@ -155,7 +155,7 @@
     <x:t xml:space="preserve">어디갔지 | API 명세서</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">API v2.2 · Issue #57 구현 기준 · 2026-09-28</x:t>
+    <x:t xml:space="preserve">API v2.3 · Issue #80 구현 기준 · 2026-09-28</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">내부 REST API</x:t>
@@ -173,7 +173,7 @@
     <x:t xml:space="preserve">상태</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">확정 · 이 문서는 Issue #57 구현을 반영한 API v2.2 확정본입니다.</x:t>
+    <x:t xml:space="preserve">확정 · 이 문서는 Issue #80 구현을 반영한 API v2.3 확정본입니다.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">유지</x:t>
@@ -209,7 +209,7 @@
     <x:t xml:space="preserve">검증</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">YAML 파싱·$ref·샘플94건·DB72컬럼 대조와 일반·포털 목록·상세 HTTP 실호출 이력 확인. Issue #57은 Mock/Fake·SQLite 집중 검증을 수행했으며 실제 OpenAI·경찰·포털·SMTP 호출과 MySQL 검증은 수행하지 않음.</x:t>
+    <x:t xml:space="preserve">YAML 파싱·$ref·샘플94건·DB72컬럼 대조와 일반·포털 목록·상세 HTTP 실호출 이력 확인. Issue #57·#80은 Mock/Fake·SQLite 집중 검증을 수행했으며 실제 OpenAI·경찰·포털·SMTP 호출과 MySQL 검증은 수행하지 않음.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">주의</x:t>
@@ -3176,10 +3176,10 @@
     <x:t xml:space="preserve">TC-11</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">AI가 후보 추가·누락·중복·key변경·순위오류·부적절한 추천이유 출력</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AI 응답 전체 폐기; 같은 최대100 후보를 규칙 기반으로 반환; UNAVAILABLE 경고; 임의 사실·후보 미표시</x:t>
+    <x:t xml:space="preserve">AI가 후보 추가·누락·중복·key변경·score오류·부적절한 추천이유 출력</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">AI 응답 전체 폐기; 같은 최대20 후보를 규칙 기반으로 반환; UNAVAILABLE 경고; 임의 사실·후보 미표시</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">TC-12</x:t>
@@ -7444,7 +7444,7 @@
         <v>포털기관 목록 2번 API ItemList</v>
       </c>
       <c r="D11" s="10" t="str">
-        <v>productNameKeyword/PRDT_NM·storagePlaceKeyword/DEP_PLACE로 포털만 조회; 일반 경찰청 호출0회; OpenAI rank/reason 반환</v>
+        <v>productNameKeyword/PRDT_NM·storagePlaceKeyword/DEP_PLACE로 포털만 조회; 일반 경찰청 호출0회; OpenAI score·서버 rank 반환</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>63</v>
@@ -7481,10 +7481,10 @@
         <v>79</v>
       </c>
       <c r="C13" s="10" t="str">
-        <v>후보1·100·101건 및 자연키 중복</v>
+        <v>후보1·20·21·72·100·101건 및 자연키 중복</v>
       </c>
       <c r="D13" s="10" t="str">
-        <v>1건 rank=1; 최대100개; 중복 제거·안정 사전축약·RESULT_LIMIT_REACHED; fdSn 문자열 보존</v>
+        <v>1건 rank=1; 최대20개; 중복 제거·결정적 사전축약·RESULT_LIMIT_REACHED; fdSn 문자열 보존</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>63</v>
@@ -7524,7 +7524,7 @@
         <v>AI timeout·429·4xx·5xx·refusal·Schema 오류 / 검색 중 동시 수정</v>
       </c>
       <c r="D15" s="10" t="str">
-        <v>timeout·408·504는504, 429는429; 기타 실패는 UNAVAILABLE+동일 집합 fallback; stale snapshot은409 ITEM_BUSY</v>
+        <v>조건 구조화 timeout·408·504는504, 429는429; 후보 평가 실패는 timeout·429 포함 201+UNAVAILABLE+동일 20건 fallback; stale snapshot은409 ITEM_BUSY</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>63</v>
@@ -9330,7 +9330,7 @@
         <v>1102</v>
       </c>
       <c r="D18" s="8" t="str">
-        <v>설명2,000·장소255·후보 문자열100~300 code point, 최종 OpenAI 요청128KiB, 후보 최대100건. 포털기관 목록 2번 결과를 자연키로 중복 제거하고 안정 축약한다.</v>
+        <v>설명2,000·장소255·후보 문자열100~300 code point, 최종 OpenAI 요청128KiB, 후보 최대20건. 포털기관 목록 2번 결과를 자연키로 중복 제거하고 결정적 축약한다.</v>
       </c>
       <c r="E18" s="8" t="str">
         <v>후보0건은 AI 미호출. API-05 성공·fallback 모두 LostItemCandidate를 저장하지 않고 persisted=false. OpenAI·외부조회는 트랜잭션 밖이며 FoundItem 원본 캐시만 마지막 짧은 트랜잭션에서 upsert. 모델은 OPENAI_MODEL=gpt-4o-mini, 자동 retry/model fallback 없음.</v>
@@ -14766,7 +14766,7 @@
         <v>5</v>
       </c>
       <c r="D29" s="15" t="str">
-        <v>atcId를 openId로 노출하고 fdSn 문자열을 보존한다. 자연키 중복 제거 후 최대 100건을 OpenAI로 랭킹한다.</v>
+        <v>atcId를 openId로 노출하고 fdSn 문자열을 보존한다. 결정적 사전 축약한 최대 20건만 OpenAI로 평가하고 rank는 서버가 부여한다.</v>
       </c>
     </row>
     <row r="30" ht="45" customHeight="1">
@@ -21149,7 +21149,7 @@
         <v>624</v>
       </c>
       <c r="F101" s="8" t="str">
-        <v>Frontend 호환용 이름. transient 결과 최대100개이며 Candidate Entity 저장을 뜻하지 않음</v>
+        <v>Frontend 호환용 이름. API-05 transient 최대20개이며 Candidate Entity 저장을 뜻하지 않음</v>
       </c>
       <c r="G101" s="8" t="s">
         <v>338</v>
@@ -26313,7 +26313,7 @@
         <v>정수</v>
       </c>
       <c r="F9" s="10" t="str">
-        <v>응답 자연키 중복 제거 후 최대100건 사전 축약</v>
+        <v>응답 자연키 중복 제거 후 최대20건 결정적 사전 축약</v>
       </c>
       <c r="G9" s="10" t="str">
         <v>https://www.data.go.kr/data/15057670/openapi.do</v>

</xml_diff>